<commit_message>
feat(F-NAR-019): ATOM-DIF.COR.001-03 Les bateaux de pomme
</commit_message>
<xml_diff>
--- a/stories/arbres/ATOM-DIF.COR.001-03.xlsx
+++ b/stories/arbres/ATOM-DIF.COR.001-03.xlsx
@@ -688,7 +688,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Nino, Mila, maman</t>
+          <t>Nino, Mila, papa, maman</t>
         </is>
       </c>
     </row>
@@ -846,7 +846,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Nino veut faire flotter des bateaux de pomme. La bassine est trop haute pour Mila. Ils la posent sur la marche et soufflent ensemble jusqu'au bord.</t>
+          <t>Une odeur de beurre monte de la pierre du jardin. Sur le bord, un éclat de bassine luit. Nino veut le bateau de pomme jusqu'au bord d'en face, maintenant. Il pousse trop fort depuis la table : la pomme s'arrête au milieu. Mila n'atteint pas. Sourire parti. Papa s'accroupit. Il refuse de foncer, pose la bassine sur la marche, souffle avec Mila. Merci vécu. Un second bateau tape le bord. Il attend. L'éclat de bassine tient.</t>
         </is>
       </c>
     </row>
@@ -1189,17 +1189,17 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>La tarte aux pommes fume encore. Elle sent le beurre. Maman l'a posée sur la pierre. La pierre est froide, sous le plat. Une pomme tombée attend dans l'herbe. Une feuille y est collée. Tu as senti la tarte, Nino ? Oui, maman. Elle est chaude. Elle va refroidir. Je veux un bateau de pomme. Dans la bassine ? Oui. En ce moment, Nino prend la pomme. Elle est collante, un peu sucrée. Maman pose une bassine d'eau. La bassine est sur la table. Mila arrive sous l'arbre. Mila est plus petite. Nino est plus grand. Ils ont des tailles différentes. Tu veux le bateau avec moi ? Oui. Mila lève les mains. La table est trop haute pour elle. Elle n'atteint pas. On pose la bassine plus bas. Maman la pose sur la marche. L'eau tremble, puis s'arrête. Vous jouez ensemble, là. On peut jouer ensemble. Nino met une feuille en voile. Mila pousse la pomme dans l'eau. La pomme tourne, tout seule. Elle fait des ronds ! Oui. On souffle ? Oui. Ils soufflent ensemble. L'eau fait de toutes petites vagues. Ça sent encore le beurre, derrière. La tarte attend. Le bateau d'abord.</t>
+          <t>Une odeur de beurre monte de la pierre. La pierre du jardin est froide, sous le plat. La tarte aux pommes fume, tiède. Elle sent le beurre, papa. Tu l'as vue, sur la pierre ? Oui, papa. Elle va refroidir, Nino. Une pomme tombée attend dans l'herbe. Une feuille y est collée, un peu sucrée. L'herbe pique un peu, sous les pieds. Une bassine d'eau attend sur la marche. Le soleil tape le bord, étroit. Un rond blanc danse dans l'eau. Sur le bord, un éclat de bassine luit. Il brille, maman. Tu le vois, sur le bord ? Oui, il brille. C'est le bord de la bassine. Je veux un bateau, maintenant ! Un bateau de pomme ? Oui, jusqu'au bord, là-bas. Jusqu'au bord d'en face ? Oui, tout de suite ! En ce moment, Nino prend la pomme. Elle est collante, un peu sucrée. Il plante la feuille, en voile. Maman pose la bassine sur la table. La table est haute, près de l'arbre. Mila arrive sous l'arbre. Elle lève les mains vers l'eau. Tu viens ? Oui. Mila se dresse sur les pointes. Ses doigts n'atteignent pas l'eau. Je n'arrive pas. Moi, je pousse ! Nino pousse trop fort, trop loin. La pomme tourne, puis s'arrête au milieu. Elle n'arrive pas. L'éclat de bassine saute près de l'eau. Le sourire de Nino disparaît. Dans sa poitrine, l'envie et l'inquiétude se bousculent. Ses épaules tombent un peu. Papa s'accroupit à la même hauteur. Tu veux le bateau jusqu'au bord ? Oui, papa. Avec Mila, Nino ? Oui. Elle n'atteint pas la table ? Non.</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>La tarte aux pommes fume encore. Elle sent le beurre. Maman l'a posée sur la pierre. La pierre est froide, sous le plat. Une pomme tombée attend dans l'herbe. Une feuille y est collée. Tu as senti la tarte, Nino ? Oui, maman. Elle est chaude. Elle va refroidir. Je veux un bateau de pomme. Dans la bassine ? Oui. En ce moment, Nino prend la pomme. Elle est collante, un peu sucrée. Maman pose une bassine d'eau. La bassine est sur la table. Mila arrive sous l'arbre. Mila est plus petite. Nino est plus grand. Ils ont des tailles différentes. Tu veux le bateau avec moi ? Oui. Mila lève les mains. La table est trop haute pour elle. Elle n'atteint pas. On pose la bassine plus bas. Maman la pose sur la marche. L'eau tremble, puis s'arrête. Vous jouez ensemble, là. On peut jouer ensemble. Nino met une feuille en voile. Mila pousse la pomme dans l'eau. La pomme tourne, tout seule. Elle fait des ronds ! Oui. On souffle ? Oui. Ils soufflent ensemble. L'eau fait de toutes petites vagues. Ça sent encore le beurre, derrière. La tarte attend. Le bateau d'abord.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Une odeur de beurre monte de la pierre. La pierre du jardin est froide, sous le plat. La tarte aux pommes fume, tiède. Elle sent le beurre, papa. Tu l'as vue, sur la pierre ? Oui, papa. Elle va refroidir, Nino. Une pomme tombée attend dans l'herbe. Une feuille y est collée, un peu sucrée. L'herbe pique un peu, sous les pieds. Une bassine d'eau attend sur la marche. Le soleil tape le bord, étroit. Un rond blanc danse dans l'eau. Sur le bord, un &lt;emphasis level="moderate"&gt;éclat de bassine&lt;/emphasis&gt; luit. Il brille, maman. Tu le vois, sur le bord ? Oui, il brille. C'est le bord de la bassine. Je veux un bateau, maintenant ! Un bateau de pomme ? Oui, jusqu'au bord, là-bas. Jusqu'au bord d'en face ? Oui, tout de suite ! En ce moment, Nino prend la pomme. Elle est collante, un peu sucrée. Il plante la feuille, en voile. Maman pose la bassine sur la table. La table est haute, près de l'arbre. Mila arrive sous l'arbre. Elle lève les mains vers l'eau. Tu viens ? Oui. Mila se dresse sur les pointes. Ses doigts n'atteignent pas l'eau. Je n'arrive pas. Moi, je pousse ! Nino pousse trop fort, trop loin. La pomme tourne, puis s'arrête au milieu. Elle n'arrive pas. L'éclat de bassine saute près de l'eau. Le sourire de Nino disparaît. Dans sa poitrine, l'envie et l'inquiétude se bousculent. Ses épaules tombent un peu. Papa s'accroupit à la même hauteur. Tu veux le bateau jusqu'au bord ? Oui, papa. Avec Mila, Nino ? Oui. Elle n'atteint pas la table ? Non.&lt;/prosody&gt;&lt;break time="500ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>Maman emmène Lila dans le jardin. Tom arrive. Tom est plus grand. Lila est plus petite. Ils ont des &lt;emphasis&gt;tailles&lt;/emphasis&gt; différentes. Un panier de pommes est posé. Lila hésite. Elle se dit que Tom atteint plus haut. Maman s'accroupit. Maman dit : les tailles différentes n'empêchent pas le jeu. On invite. On joue ensemble. Lila va vers Tom. Elle dit : tu veux le panier avec moi. Tom dit : oui. Tom tend une pomme tout près. Lila la pose. Ils font un tas. Parfois Tom pose plus haut. Parfois Lila pose tout bas. Les deux façons marchent. Plus tard, ils rentrent au salon. Maman sort des cerceaux. Tom enfile le grand. Lila enfile le petit. Lila se souvient. Elle invite. Tom dit oui. Ils font rouler les cerceaux. Maman dit : au jardin, puis ici. C'est la même leçon. Petit ou grand, on invite. On joue ensemble. Lila et Tom tapent dans leurs mains. Les tailles différentes sont encore là. Le jeu aussi. [pause]</t>
+          <t>Une odeur de beurre monte de la pierre. La pierre du jardin est froide, sous le plat. La tarte aux pommes fume, tiède. Elle sent le beurre, papa. Tu l'as vue, sur la pierre ? Oui, papa. Elle va refroidir, Nino. Une pomme tombée attend dans l'herbe. Une feuille y est collée, un peu sucrée. L'herbe pique un peu, sous les pieds. Une bassine d'eau attend sur la marche. Le soleil tape le bord, étroit. Un rond blanc danse dans l'eau. Sur le bord, un &lt;emphasis&gt;éclat de bassine&lt;/emphasis&gt; luit. Il brille, maman. Tu le vois, sur le bord ? Oui, il brille. C'est le bord de la bassine. Je veux un bateau, maintenant ! Un bateau de pomme ? Oui, jusqu'au bord, là-bas. Jusqu'au bord d'en face ? Oui, tout de suite ! En ce moment, Nino prend la pomme. Elle est collante, un peu sucrée. Il plante la feuille, en voile. Maman pose la bassine sur la table. La table est haute, près de l'arbre. Mila arrive sous l'arbre. Elle lève les mains vers l'eau. Tu viens ? Oui. Mila se dresse sur les pointes. Ses doigts n'atteignent pas l'eau. Je n'arrive pas. Moi, je pousse ! Nino pousse trop fort, trop loin. La pomme tourne, puis s'arrête au milieu. Elle n'arrive pas. L'éclat de bassine saute près de l'eau. Le sourire de Nino disparaît. Dans sa poitrine, l'envie et l'inquiétude se bousculent. Ses épaules tombent un peu. Papa s'accroupit à la même hauteur. Tu veux le bateau jusqu'au bord ? Oui, papa. Avec Mila, Nino ? Oui. Elle n'atteint pas la table ? Non. [pause]</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr"/>
@@ -1246,7 +1246,7 @@
         </is>
       </c>
       <c r="Y2" s="2" t="n">
-        <v>148</v>
+        <v>142</v>
       </c>
       <c r="Z2" s="2" t="inlineStr">
         <is>
@@ -1254,10 +1254,10 @@
         </is>
       </c>
       <c r="AA2" s="2" t="n">
-        <v>0.96</v>
+        <v>0.98</v>
       </c>
       <c r="AB2" s="2" t="n">
-        <v>1.22</v>
+        <v>1.12</v>
       </c>
       <c r="AC2" s="2" t="inlineStr">
         <is>
@@ -1280,30 +1280,30 @@
       </c>
       <c r="AH2" s="2" t="inlineStr">
         <is>
-          <t>tailles</t>
+          <t>éclat de bassine</t>
         </is>
       </c>
       <c r="AI2" s="2" t="n">
         <v>0</v>
       </c>
       <c r="AJ2" s="2" t="n">
-        <v>400</v>
+        <v>500</v>
       </c>
       <c r="AK2" s="2" t="n">
-        <v>280</v>
+        <v>260</v>
       </c>
       <c r="AL2" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>warm</t>
         </is>
       </c>
       <c r="AM2" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>storytelling</t>
         </is>
       </c>
       <c r="AN2" s="2" t="n">
-        <v>0.333</v>
+        <v>0.36</v>
       </c>
       <c r="AO2" s="2" t="inlineStr"/>
       <c r="AP2" s="2" t="inlineStr">
@@ -1312,10 +1312,10 @@
         </is>
       </c>
       <c r="AQ2" s="2" t="n">
-        <v>0.96</v>
+        <v>0.98</v>
       </c>
       <c r="AR2" s="2" t="n">
-        <v>0.96</v>
+        <v>0.98</v>
       </c>
       <c r="AS2" s="2" t="n">
         <v>100</v>
@@ -1326,52 +1326,68 @@
       <c r="AU2" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="AV2" s="2" t="inlineStr"/>
+      <c r="AV2" s="2" t="inlineStr">
+        <is>
+          <t>arc=installation; intention=émerveiller puis tendre; emotion=impatience puis découragement; intensite=2; destinataire=enfant; sous_texte=il_veut_le_bateau_jusqu_au_bord_maintenant; tempo=naturel puis resserré; sourire=léger puis aucun; respiration=ample puis retenue</t>
+        </is>
+      </c>
       <c r="AW2" t="inlineStr">
         <is>
-          <t>narrateur|La tarte aux pommes fume encore.
-narrateur|Elle sent le beurre.
-narrateur|Maman l'a posée sur la pierre.
-narrateur|La pierre est froide, sous le plat.
+          <t>narrateur|Une odeur de beurre monte de la pierre.
+narrateur|La pierre du jardin est froide, sous le plat.
+narrateur|La tarte aux pommes fume, tiède.
+enfant-m|Elle sent le beurre, papa.
+papa|Tu l'as vue, sur la pierre ?
+enfant-m|Oui, papa.
+maman|Elle va refroidir, Nino.
 narrateur|Une pomme tombée attend dans l'herbe.
-narrateur|Une feuille y est collée.
-maman|Tu as senti la tarte, Nino ?
-enfant-m|Oui, maman.
-enfant-m|Elle est chaude.
-maman|Elle va refroidir.
-enfant-m|Je veux un bateau de pomme.
-maman|Dans la bassine ?
-enfant-m|Oui.
+narrateur|Une feuille y est collée, un peu sucrée.
+narrateur|L'herbe pique un peu, sous les pieds.
+narrateur|Une bassine d'eau attend sur la marche.
+narrateur|Le soleil tape le bord, étroit.
+narrateur|Un rond blanc danse dans l'eau.
+narrateur|Sur le bord, un éclat de bassine luit.
+enfant-m|Il brille, maman.
+maman|Tu le vois, sur le bord ?
+enfant-m|Oui, il brille.
+papa|C'est le bord de la bassine.
+enfant-m|Je veux un bateau, maintenant !
+maman|Un bateau de pomme ?
+enfant-m|Oui, jusqu'au bord, là-bas.
+papa|Jusqu'au bord d'en face ?
+enfant-m|Oui, tout de suite !
 narrateur|En ce moment, Nino prend la pomme.
 narrateur|Elle est collante, un peu sucrée.
-narrateur|Maman pose une bassine d'eau.
-narrateur|La bassine est sur la table.
+narrateur|Il plante la feuille, en voile.
+narrateur|Maman pose la bassine sur la table.
+narrateur|La table est haute, près de l'arbre.
 narrateur|Mila arrive sous l'arbre.
-narrateur|Mila est plus petite.
-narrateur|Nino est plus grand.
-narrateur|Ils ont des tailles différentes.
-enfant-m|Tu veux le bateau avec moi ?
+narrateur|Elle lève les mains vers l'eau.
+enfant-m|Tu viens ?
 copine|Oui.
-narrateur|Mila lève les mains.
-narrateur|La table est trop haute pour elle.
-enfant-m|Elle n'atteint pas.
-maman|On pose la bassine plus bas.
-narrateur|Maman la pose sur la marche.
-narrateur|L'eau tremble, puis s'arrête.
-maman|Vous jouez ensemble, là.
-maman|On peut jouer ensemble.
-narrateur|Nino met une feuille en voile.
-narrateur|Mila pousse la pomme dans l'eau.
-narrateur|La pomme tourne, tout seule.
-enfant-m|Elle fait des ronds !
-maman|Oui.
-copine|On souffle ?
+narrateur|Mila se dresse sur les pointes.
+narrateur|Ses doigts n'atteignent pas l'eau.
+copine|Je n'arrive pas.
+enfant-m|Moi, je pousse !
+narrateur|Nino pousse trop fort, trop loin.
+narrateur|La pomme tourne, puis s'arrête au milieu.
+enfant-m|Elle n'arrive pas.
+narrateur|L'éclat de bassine saute près de l'eau.
+narrateur|Le sourire de Nino disparaît.
+narrateur|Dans sa poitrine, l'envie et l'inquiétude se bousculent.
+narrateur|Ses épaules tombent un peu.
+narrateur|Papa s'accroupit à la même hauteur.
+papa|Tu veux le bateau jusqu'au bord ?
+enfant-m|Oui, papa.
+maman|Avec Mila, Nino ?
 enfant-m|Oui.
-narrateur|Ils soufflent ensemble.
-narrateur|L'eau fait de toutes petites vagues.
-narrateur|Ça sent encore le beurre, derrière.
-maman|La tarte attend.
-enfant-m|Le bateau d'abord.</t>
+papa|Elle n'atteint pas la table ?
+enfant-m|Non.</t>
+        </is>
+      </c>
+      <c r="AX2" t="inlineStr">
+        <is>
+          <t>tarte,pierre,bassine</t>
         </is>
       </c>
     </row>
@@ -1403,12 +1419,12 @@
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>Nino est plus grand. Mila est plus petite. Que font-ils ?</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="medium"&gt;Nino est plus grand. &lt;emphasis level="moderate"&gt;Mila&lt;/emphasis&gt; est plus petite. Que font-ils ?&lt;/prosody&gt;&lt;break time="700ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>Lila est plus petite. Tom est plus grand. Que font-ils ?</t>
+          <t>&lt;soft&gt;&lt;slow&gt;Nino est plus grand. &lt;emphasis&gt;Mila&lt;/emphasis&gt; est plus petite. Que font-ils ?&lt;/slow&gt;&lt;/soft&gt; [pause]</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -1418,7 +1434,7 @@
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>jouer ensemble | ensemble | ils jouent | inviter | le panier</t>
+          <t>jouer ensemble | ensemble | ils jouent | on joue | souffler ensemble</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
@@ -1471,7 +1487,7 @@
         </is>
       </c>
       <c r="Y3" s="2" t="n">
-        <v>130</v>
+        <v>120</v>
       </c>
       <c r="Z3" s="2" t="inlineStr">
         <is>
@@ -1479,10 +1495,10 @@
         </is>
       </c>
       <c r="AA3" s="2" t="n">
-        <v>0.9</v>
+        <v>0.86</v>
       </c>
       <c r="AB3" s="2" t="n">
-        <v>1.24</v>
+        <v>1.27</v>
       </c>
       <c r="AC3" s="2" t="inlineStr">
         <is>
@@ -1497,34 +1513,38 @@
       <c r="AE3" s="2" t="inlineStr"/>
       <c r="AF3" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>soft</t>
         </is>
       </c>
       <c r="AG3" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="AH3" s="2" t="inlineStr"/>
+        <v>-2</v>
+      </c>
+      <c r="AH3" s="2" t="inlineStr">
+        <is>
+          <t>Mila</t>
+        </is>
+      </c>
       <c r="AI3" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ3" s="2" t="n">
-        <v>250</v>
+        <v>700</v>
       </c>
       <c r="AK3" s="2" t="n">
-        <v>280</v>
+        <v>320</v>
       </c>
       <c r="AL3" s="2" t="inlineStr">
         <is>
-          <t>warm</t>
+          <t>focused</t>
         </is>
       </c>
       <c r="AM3" s="2" t="inlineStr">
         <is>
-          <t>rise</t>
+          <t>rising</t>
         </is>
       </c>
       <c r="AN3" s="2" t="n">
-        <v>0.333</v>
+        <v>0.32</v>
       </c>
       <c r="AO3" s="2" t="inlineStr"/>
       <c r="AP3" s="2" t="inlineStr">
@@ -1533,23 +1553,23 @@
         </is>
       </c>
       <c r="AQ3" s="2" t="n">
-        <v>0.9</v>
+        <v>0.86</v>
       </c>
       <c r="AR3" s="2" t="n">
-        <v>0.9</v>
+        <v>0.86</v>
       </c>
       <c r="AS3" s="2" t="n">
-        <v>100</v>
+        <v>82</v>
       </c>
       <c r="AT3" s="2" t="n">
         <v>50</v>
       </c>
       <c r="AU3" s="2" t="n">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="AV3" s="2" t="inlineStr">
         <is>
-          <t>question d'écoute, ne change pas le cours</t>
+          <t>arc=indice; intention=faire_deviner; emotion=attention; intensite=1; destinataire=enfant; sous_texte=plus_grand_plus_petite_ils_jouent_ensemble; tempo=suspendu; sourire=aucun; respiration=courte_avant_question</t>
         </is>
       </c>
       <c r="AW3" t="inlineStr">
@@ -1583,17 +1603,17 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Le bateau arrive au bord. Mila le rattrape tout bas. Nino en prépare un autre. Une feuille verte, une pomme jaune. Deux bateaux, maintenant. Oui. Les deux façons marchent. Parfois Nino pousse plus loin. Parfois Mila pousse tout près. Les pommes se croisent. La mienne a tourné ! La mienne aussi. Vous avez des tailles différentes. Et vous jouez ensemble. Le bateau a bien flotté ? Oui, maman. Une goutte tombe de la feuille. Elle fait un rond dans l'eau. La tarte ne fume plus. Elle sent encore le beurre. Elle est prête ? Presque. Un bateau encore, si vous voulez. Encore un.</t>
+          <t>Nino veut pousser, d'un coup. Nino refuse de foncer. Personne ne parle. Il observe l'eau, un instant. Il écoute le jardin, près de la pierre. Sur le bord, l'éclat de bassine revient. On pose la bassine, plus bas. Sur la marche ? Oui, papa. Papa pose la bassine sur la marche. L'eau tremble, puis s'arrête. Mila touche l'eau, du bout des doigts. Elle est froide. On souffle ? Oui. Ils soufflent du même côté de l'eau. La pomme glisse, lente, vers le bord. Elle arrive ! Je la tiens. Mila rattrape la pomme, près d'elle. Nino reste de son côté, plus haut. Merci, Nino. Papa a regardé jusqu'au bout. Le ventre de Nino se desserre. Un autre bateau ? La tarte attend un peu. Le bateau d'abord. Tes pieds sont sur la marche ? Oui, maman. Et Mila ? Moi aussi.</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Le bateau arrive au bord. Mila le rattrape tout bas. Nino en prépare un autre. Une feuille verte, une pomme jaune. Deux bateaux, maintenant. Oui. Les deux façons marchent. Parfois Nino pousse plus loin. Parfois Mila pousse tout près. Les pommes se croisent. La mienne a tourné ! La mienne aussi. Vous avez des tailles différentes. Et vous jouez ensemble. Le bateau a bien flotté ? Oui, maman. Une goutte tombe de la feuille. Elle fait un rond dans l'eau. La tarte ne fume plus. Elle sent encore le beurre. Elle est prête ? Presque. Un bateau encore, si vous voulez. Encore un.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Nino veut pousser, d'un coup. Nino refuse de foncer. Personne ne parle. Il observe l'eau, un instant. Il écoute le jardin, près de la pierre. Sur le bord, l'éclat de bassine revient. On pose la bassine, plus bas. Sur la &lt;emphasis level="moderate"&gt;marche&lt;/emphasis&gt; ? Oui, papa. Papa pose la bassine sur la marche. L'eau tremble, puis s'arrête. Mila touche l'eau, du bout des doigts. Elle est froide. On souffle ? Oui. Ils soufflent du même côté de l'eau. La pomme glisse, lente, vers le bord. Elle arrive ! Je la tiens. Mila rattrape la pomme, près d'elle. Nino reste de son côté, plus haut. Merci, Nino. Papa a regardé jusqu'au bout. Le ventre de Nino se desserre. Un autre bateau ? La tarte attend un peu. Le bateau d'abord. Tes pieds sont sur la marche ? Oui, maman. Et Mila ? Moi aussi.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>Lila a invité. Tom a tendu la pomme tout près. Ils ont des &lt;emphasis&gt;tailles&lt;/emphasis&gt; différentes. Ils ont joué ensemble. [pause]</t>
+          <t>Nino veut pousser, d'un coup. Nino refuse de foncer. Personne ne parle. Il observe l'eau, un instant. Il écoute le jardin, près de la pierre. Sur le bord, l'éclat de bassine revient. On pose la bassine, plus bas. Sur la &lt;emphasis&gt;marche&lt;/emphasis&gt; ? Oui, papa. Papa pose la bassine sur la marche. L'eau tremble, puis s'arrête. Mila touche l'eau, du bout des doigts. Elle est froide. On souffle ? Oui. Ils soufflent du même côté de l'eau. La pomme glisse, lente, vers le bord. Elle arrive ! Je la tiens. Mila rattrape la pomme, près d'elle. Nino reste de son côté, plus haut. Merci, Nino. Papa a regardé jusqu'au bout. Le ventre de Nino se desserre. Un autre bateau ? La tarte attend un peu. Le bateau d'abord. Tes pieds sont sur la marche ? Oui, maman. Et Mila ? Moi aussi. [pause]</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr"/>
@@ -1640,7 +1660,7 @@
         </is>
       </c>
       <c r="Y4" s="2" t="n">
-        <v>148</v>
+        <v>140</v>
       </c>
       <c r="Z4" s="2" t="inlineStr">
         <is>
@@ -1648,10 +1668,10 @@
         </is>
       </c>
       <c r="AA4" s="2" t="n">
-        <v>0.96</v>
+        <v>0.97</v>
       </c>
       <c r="AB4" s="2" t="n">
-        <v>1.22</v>
+        <v>1.14</v>
       </c>
       <c r="AC4" s="2" t="inlineStr">
         <is>
@@ -1674,30 +1694,30 @@
       </c>
       <c r="AH4" s="2" t="inlineStr">
         <is>
-          <t>tailles</t>
+          <t>marche</t>
         </is>
       </c>
       <c r="AI4" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ4" s="2" t="n">
-        <v>450</v>
+        <v>560</v>
       </c>
       <c r="AK4" s="2" t="n">
-        <v>280</v>
+        <v>270</v>
       </c>
       <c r="AL4" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>bright</t>
         </is>
       </c>
       <c r="AM4" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>falling</t>
         </is>
       </c>
       <c r="AN4" s="2" t="n">
-        <v>0.333</v>
+        <v>0.35</v>
       </c>
       <c r="AO4" s="2" t="inlineStr"/>
       <c r="AP4" s="2" t="inlineStr">
@@ -1706,10 +1726,10 @@
         </is>
       </c>
       <c r="AQ4" s="2" t="n">
-        <v>0.96</v>
+        <v>0.97</v>
       </c>
       <c r="AR4" s="2" t="n">
-        <v>0.96</v>
+        <v>0.97</v>
       </c>
       <c r="AS4" s="2" t="n">
         <v>100</v>
@@ -1722,35 +1742,47 @@
       </c>
       <c r="AV4" s="2" t="inlineStr">
         <is>
-          <t>confirmation ; le moteur peut dire engine_ok/near avant ce chunk</t>
+          <t>arc=résolution; intention=faire_vivre_le_geste; emotion=retenue puis fierté_calme; intensite=2; destinataire=enfant; sous_texte=bassine_sur_la_marche_ils_soufflent; tempo=naturel; sourire=léger; respiration=relâchée</t>
         </is>
       </c>
       <c r="AW4" t="inlineStr">
         <is>
-          <t>narrateur|Le bateau arrive au bord.
-narrateur|Mila le rattrape tout bas.
-narrateur|Nino en prépare un autre.
-narrateur|Une feuille verte, une pomme jaune.
-enfant-m|Deux bateaux, maintenant.
-maman|Oui.
-maman|Les deux façons marchent.
-narrateur|Parfois Nino pousse plus loin.
-narrateur|Parfois Mila pousse tout près.
-narrateur|Les pommes se croisent.
-copine|La mienne a tourné !
-enfant-m|La mienne aussi.
-maman|Vous avez des tailles différentes.
-maman|Et vous jouez ensemble.
-maman|Le bateau a bien flotté ?
+          <t>narrateur|Nino veut pousser, d'un coup.
+narrateur|Nino refuse de foncer.
+narrateur|Personne ne parle.
+narrateur|Il observe l'eau, un instant.
+narrateur|Il écoute le jardin, près de la pierre.
+narrateur|Sur le bord, l'éclat de bassine revient.
+enfant-m|On pose la bassine, plus bas.
+papa|Sur la marche ?
+enfant-m|Oui, papa.
+narrateur|Papa pose la bassine sur la marche.
+narrateur|L'eau tremble, puis s'arrête.
+narrateur|Mila touche l'eau, du bout des doigts.
+copine|Elle est froide.
+enfant-m|On souffle ?
+copine|Oui.
+narrateur|Ils soufflent du même côté de l'eau.
+narrateur|La pomme glisse, lente, vers le bord.
+enfant-m|Elle arrive !
+copine|Je la tiens.
+narrateur|Mila rattrape la pomme, près d'elle.
+narrateur|Nino reste de son côté, plus haut.
+papa|Merci, Nino.
+narrateur|Papa a regardé jusqu'au bout.
+narrateur|Le ventre de Nino se desserre.
+enfant-m|Un autre bateau ?
+maman|La tarte attend un peu.
+enfant-m|Le bateau d'abord.
+maman|Tes pieds sont sur la marche ?
 enfant-m|Oui, maman.
-narrateur|Une goutte tombe de la feuille.
-narrateur|Elle fait un rond dans l'eau.
-narrateur|La tarte ne fume plus.
-narrateur|Elle sent encore le beurre.
-enfant-m|Elle est prête ?
-maman|Presque.
-maman|Un bateau encore, si vous voulez.
-copine|Encore un.</t>
+papa|Et Mila ?
+copine|Moi aussi.</t>
+        </is>
+      </c>
+      <c r="AX4" t="inlineStr">
+        <is>
+          <t>eau,pomme</t>
         </is>
       </c>
     </row>
@@ -1777,17 +1809,17 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>On range les pommes sur l'assiette ? Oui. Nino pose une pomme. Mila pose l'autre. Les voiles de feuilles restent à côté. Tu as fini de poser les bateaux ? Oui, maman. Maman vide la bassine, tout bas. L'eau part dans l'herbe. À demain. À demain. La pierre sous la tarte est sèche. Le jardin sent le fruit et le beurre.</t>
+          <t>Nino prépare une autre pomme. Une feuille verte tient, collée. Celle-là, plus loin ! Il pousse trop vite, du haut de la marche. L'eau saute contre le bord. La pomme tape le bord, puis revient. Oh. Mila retire les mains. Non. Le sourire ne revient pas. Nino veut rattraper, d'un coup. Nino refuse de foncer. Ses épaules se serrent un peu. Ça tape, dans sa poitrine. Personne ne dit la suite. Il regarde le bord, il écoute l'eau. Un oiseau passe, loin. On souffle, Mila ? Mila ne dit rien. Elle garde les mains sur ses genoux. D'accord. Nino attend. Plus tard. Oui. La pomme se cale, sans tourner. Mila avance un doigt. Elle pousse près d'elle, puis s'arrête. D'accord. Ils soufflent, chacun de son bord. Les deux pommes se croisent. La mienne a tourné ! La mienne aussi. La tarte ne fume plus. Elle est prête ? Presque. Tes mains sont dans l'eau ? Oui, papa.</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>On range les pommes sur l'assiette ? Oui. Nino pose une pomme. Mila pose l'autre. Les voiles de feuilles restent à côté. Tu as fini de poser les bateaux ? Oui, maman. Maman vide la bassine, tout bas. L'eau part dans l'herbe. À demain. À demain. La pierre sous la tarte est sèche. Le jardin sent le fruit et le beurre.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Nino prépare une autre &lt;emphasis level="moderate"&gt;pomme&lt;/emphasis&gt;. Une feuille verte tient, collée. Celle-là, plus loin ! Il pousse trop vite, du haut de la marche. L'eau saute contre le bord. La pomme tape le bord, puis revient. Oh. Mila retire les mains. Non. Le sourire ne revient pas. Nino veut rattraper, d'un coup. Nino refuse de foncer. Ses épaules se serrent un peu. Ça tape, dans sa poitrine. Personne ne dit la suite. Il regarde le bord, il écoute l'eau. Un oiseau passe, loin. On souffle, Mila ? Mila ne dit rien. Elle garde les mains sur ses genoux. D'accord. Nino attend. Plus tard. Oui. La pomme se cale, sans tourner. Mila avance un doigt. Elle pousse près d'elle, puis s'arrête. D'accord. Ils soufflent, chacun de son bord. Les deux pommes se croisent. La mienne a tourné ! La mienne aussi. La tarte ne fume plus. Elle est prête ? Presque. Tes mains sont dans l'eau ? Oui, papa.&lt;/prosody&gt;&lt;break time="420ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>Maman range les cerceaux. Lila et Tom se disent à de&lt;emphasis&gt;main&lt;/emphasis&gt;. [pause]</t>
+          <t>Nino prépare une autre &lt;emphasis&gt;pomme&lt;/emphasis&gt;. Une feuille verte tient, collée. Celle-là, plus loin ! Il pousse trop vite, du haut de la marche. L'eau saute contre le bord. La pomme tape le bord, puis revient. Oh. Mila retire les mains. Non. Le sourire ne revient pas. Nino veut rattraper, d'un coup. Nino refuse de foncer. Ses épaules se serrent un peu. Ça tape, dans sa poitrine. Personne ne dit la suite. Il regarde le bord, il écoute l'eau. Un oiseau passe, loin. On souffle, Mila ? Mila ne dit rien. Elle garde les mains sur ses genoux. D'accord. Nino attend. Plus tard. Oui. La pomme se cale, sans tourner. Mila avance un doigt. Elle pousse près d'elle, puis s'arrête. D'accord. Ils soufflent, chacun de son bord. Les deux pommes se croisent. La mienne a tourné ! La mienne aussi. La tarte ne fume plus. Elle est prête ? Presque. Tes mains sont dans l'eau ? Oui, papa. [pause]</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr"/>
@@ -1834,7 +1866,7 @@
         </is>
       </c>
       <c r="Y5" s="2" t="n">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="Z5" s="2" t="inlineStr">
         <is>
@@ -1842,10 +1874,10 @@
         </is>
       </c>
       <c r="AA5" s="2" t="n">
-        <v>0.96</v>
+        <v>1</v>
       </c>
       <c r="AB5" s="2" t="n">
-        <v>1.22</v>
+        <v>1.1</v>
       </c>
       <c r="AC5" s="2" t="inlineStr">
         <is>
@@ -1868,30 +1900,30 @@
       </c>
       <c r="AH5" s="2" t="inlineStr">
         <is>
-          <t>main</t>
+          <t>pomme</t>
         </is>
       </c>
       <c r="AI5" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ5" s="2" t="n">
-        <v>450</v>
+        <v>420</v>
       </c>
       <c r="AK5" s="2" t="n">
-        <v>280</v>
+        <v>250</v>
       </c>
       <c r="AL5" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>lively</t>
         </is>
       </c>
       <c r="AM5" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>dynamic</t>
         </is>
       </c>
       <c r="AN5" s="2" t="n">
-        <v>0.333</v>
+        <v>0.37</v>
       </c>
       <c r="AO5" s="2" t="inlineStr"/>
       <c r="AP5" s="2" t="inlineStr">
@@ -1900,10 +1932,10 @@
         </is>
       </c>
       <c r="AQ5" s="2" t="n">
-        <v>0.96</v>
+        <v>1</v>
       </c>
       <c r="AR5" s="2" t="n">
-        <v>0.96</v>
+        <v>1</v>
       </c>
       <c r="AS5" s="2" t="n">
         <v>100</v>
@@ -1914,22 +1946,55 @@
       <c r="AU5" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="AV5" s="2" t="inlineStr"/>
+      <c r="AV5" s="2" t="inlineStr">
+        <is>
+          <t>arc=action; intention=entraîner; emotion=élan puis prudence; intensite=2; destinataire=enfant; sous_texte=il_refuse_de_pousser_trop_vite_du_haut; tempo=vif puis posé; sourire=léger; respiration=courte</t>
+        </is>
+      </c>
       <c r="AW5" t="inlineStr">
         <is>
-          <t>maman|On range les pommes sur l'assiette ?
+          <t>narrateur|Nino prépare une autre pomme.
+narrateur|Une feuille verte tient, collée.
+enfant-m|Celle-là, plus loin !
+narrateur|Il pousse trop vite, du haut de la marche.
+narrateur|L'eau saute contre le bord.
+narrateur|La pomme tape le bord, puis revient.
+enfant-m|Oh.
+narrateur|Mila retire les mains.
+copine|Non.
+narrateur|Le sourire ne revient pas.
+narrateur|Nino veut rattraper, d'un coup.
+narrateur|Nino refuse de foncer.
+narrateur|Ses épaules se serrent un peu.
+narrateur|Ça tape, dans sa poitrine.
+narrateur|Personne ne dit la suite.
+narrateur|Il regarde le bord, il écoute l'eau.
+narrateur|Un oiseau passe, loin.
+enfant-m|On souffle, Mila ?
+narrateur|Mila ne dit rien.
+narrateur|Elle garde les mains sur ses genoux.
+enfant-m|D'accord.
+narrateur|Nino attend.
+copine|Plus tard.
 enfant-m|Oui.
-narrateur|Nino pose une pomme.
-narrateur|Mila pose l'autre.
-narrateur|Les voiles de feuilles restent à côté.
-maman|Tu as fini de poser les bateaux ?
-enfant-m|Oui, maman.
-narrateur|Maman vide la bassine, tout bas.
-narrateur|L'eau part dans l'herbe.
-copine|À demain.
-enfant-m|À demain.
-narrateur|La pierre sous la tarte est sèche.
-narrateur|Le jardin sent le fruit et le beurre.</t>
+narrateur|La pomme se cale, sans tourner.
+narrateur|Mila avance un doigt.
+narrateur|Elle pousse près d'elle, puis s'arrête.
+enfant-m|D'accord.
+narrateur|Ils soufflent, chacun de son bord.
+narrateur|Les deux pommes se croisent.
+copine|La mienne a tourné !
+enfant-m|La mienne aussi.
+maman|La tarte ne fume plus.
+enfant-m|Elle est prête ?
+maman|Presque.
+papa|Tes mains sont dans l'eau ?
+enfant-m|Oui, papa.</t>
+        </is>
+      </c>
+      <c r="AX5" t="inlineStr">
+        <is>
+          <t>feuille,eau</t>
         </is>
       </c>
     </row>
@@ -1956,17 +2021,17 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>Les bateaux ont flotté. On a joué ensemble. Bravo, Nino. La tarte attend encore un peu.</t>
+          <t>Ils restent près de la marche. Les voiles de feuilles restent mouillées. L'éclat est là, papa. Tu le vois sur le bord ? Oui, papa. On est bien, ici. La tarte sent le beurre, plus légère. Mes bateaux ont flotté. Jusqu'au bord, Nino. Oui, maman. Nino pose la joue près du bord. Le bord est tiède, un peu. C'est tiède. Tu le sens sur tes joues ? Oui, il est tiède. Une feuille porte une goutte d'eau. Dehors, le jardin s'endort. L'éclat de bassine tient sur le bord.</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>Les bateaux ont flotté. On a joué ensemble. Bravo, Nino. La tarte attend encore un peu.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Ils restent près de la marche. Les voiles de feuilles restent mouillées. L'éclat est là, papa. Tu le vois sur le bord ? Oui, papa. On est bien, ici. La tarte sent le beurre, plus légère. Mes bateaux ont flotté. Jusqu'au bord, Nino. Oui, maman. Nino pose la joue près du bord. Le bord est tiède, un peu. C'est tiède. Tu le sens sur tes joues ? Oui, il est tiède. Une feuille porte une goutte d'eau. Dehors, le jardin s'endort. L'&lt;emphasis level="moderate"&gt;éclat de bassine&lt;/emphasis&gt; tient sur le bord.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>&lt;lower-pitch&gt;&lt;soft&gt;L'histoire est finie.&lt;/soft&gt;&lt;/lower-pitch&gt; [pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Ils restent près de la marche. Les voiles de feuilles restent mouillées. L'éclat est là, papa. Tu le vois sur le bord ? Oui, papa. On est bien, ici. La tarte sent le beurre, plus légère. Mes bateaux ont flotté. Jusqu'au bord, Nino. Oui, maman. Nino pose la joue près du bord. Le bord est tiède, un peu. C'est tiède. Tu le sens sur tes joues ? Oui, il est tiède. Une feuille porte une goutte d'eau. Dehors, le jardin s'endort. L'&lt;emphasis&gt;éclat de bassine&lt;/emphasis&gt; tient sur le bord.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr"/>
@@ -2013,15 +2078,15 @@
         </is>
       </c>
       <c r="Y6" s="2" t="n">
-        <v>136</v>
+        <v>118</v>
       </c>
       <c r="Z6" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>slow</t>
         </is>
       </c>
       <c r="AA6" s="2" t="n">
-        <v>0.92</v>
+        <v>0.85</v>
       </c>
       <c r="AB6" s="2" t="n">
         <v>1.28</v>
@@ -2033,12 +2098,12 @@
       </c>
       <c r="AD6" s="2" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>-2st</t>
         </is>
       </c>
       <c r="AE6" s="2" t="inlineStr">
         <is>
-          <t>lower-pitch</t>
+          <t>low-pitch</t>
         </is>
       </c>
       <c r="AF6" s="2" t="inlineStr">
@@ -2047,17 +2112,21 @@
         </is>
       </c>
       <c r="AG6" s="2" t="n">
-        <v>-2</v>
-      </c>
-      <c r="AH6" s="2" t="inlineStr"/>
+        <v>-3</v>
+      </c>
+      <c r="AH6" s="2" t="inlineStr">
+        <is>
+          <t>éclat de bassine</t>
+        </is>
+      </c>
       <c r="AI6" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ6" s="2" t="n">
-        <v>600</v>
+        <v>900</v>
       </c>
       <c r="AK6" s="2" t="n">
-        <v>280</v>
+        <v>340</v>
       </c>
       <c r="AL6" s="2" t="inlineStr">
         <is>
@@ -2066,11 +2135,11 @@
       </c>
       <c r="AM6" s="2" t="inlineStr">
         <is>
-          <t>fall</t>
+          <t>falling</t>
         </is>
       </c>
       <c r="AN6" s="2" t="n">
-        <v>0.333</v>
+        <v>0.31</v>
       </c>
       <c r="AO6" s="2" t="inlineStr"/>
       <c r="AP6" s="2" t="inlineStr">
@@ -2079,27 +2148,50 @@
         </is>
       </c>
       <c r="AQ6" s="2" t="n">
-        <v>0.92</v>
+        <v>0.85</v>
       </c>
       <c r="AR6" s="2" t="n">
-        <v>0.92</v>
+        <v>0.85</v>
       </c>
       <c r="AS6" s="2" t="n">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="AT6" s="2" t="n">
-        <v>35</v>
+        <v>42</v>
       </c>
       <c r="AU6" s="2" t="n">
-        <v>8</v>
-      </c>
-      <c r="AV6" s="2" t="inlineStr"/>
+        <v>12</v>
+      </c>
+      <c r="AV6" s="2" t="inlineStr">
+        <is>
+          <t>arc=retour; intention=refermer; emotion=tendresse et fierté_calme; intensite=1; destinataire=enfant; sous_texte=l_eclat_du_debut_tient_sur_le_bord; tempo=posé; sourire=léger; respiration=ample</t>
+        </is>
+      </c>
       <c r="AW6" t="inlineStr">
         <is>
-          <t>enfant-m|Les bateaux ont flotté.
-enfant-m|On a joué ensemble.
-maman|Bravo, Nino.
-narrateur|La tarte attend encore un peu.</t>
+          <t>narrateur|Ils restent près de la marche.
+narrateur|Les voiles de feuilles restent mouillées.
+enfant-m|L'éclat est là, papa.
+papa|Tu le vois sur le bord ?
+enfant-m|Oui, papa.
+maman|On est bien, ici.
+narrateur|La tarte sent le beurre, plus légère.
+enfant-m|Mes bateaux ont flotté.
+maman|Jusqu'au bord, Nino.
+enfant-m|Oui, maman.
+narrateur|Nino pose la joue près du bord.
+narrateur|Le bord est tiède, un peu.
+enfant-m|C'est tiède.
+papa|Tu le sens sur tes joues ?
+enfant-m|Oui, il est tiède.
+narrateur|Une feuille porte une goutte d'eau.
+narrateur|Dehors, le jardin s'endort.
+narrateur|L'éclat de bassine tient sur le bord.</t>
+        </is>
+      </c>
+      <c r="AX6" t="inlineStr">
+        <is>
+          <t>tarte</t>
         </is>
       </c>
     </row>
@@ -2120,7 +2212,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A11"/>
+  <dimension ref="A1:A12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -2198,6 +2290,13 @@
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
+        <is>
+          <t>F-NAR-008 récit, pas une leçon en puces</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
         <is>
           <t>F-NAR-008 récit, pas une leçon en puces</t>
         </is>

</xml_diff>